<commit_message>
Add some stuffs, remove some stuffs before using SpringBoot
</commit_message>
<xml_diff>
--- a/src/main/webapp/images/Product_Corrected.xlsx
+++ b/src/main/webapp/images/Product_Corrected.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="103">
   <si>
     <t>ProductID</t>
   </si>
@@ -56,6 +56,9 @@
     <t>Áo phông nữ Cotton USA basic dáng suông</t>
   </si>
   <si>
+    <t>Việt Tiến</t>
+  </si>
+  <si>
     <t>3TS26C001-SW001</t>
   </si>
   <si>
@@ -96,6 +99,9 @@
   </si>
   <si>
     <t>Áo Polo</t>
+  </si>
+  <si>
+    <t>Owen</t>
   </si>
   <si>
     <t>8TP26S005-SK010</t>
@@ -325,10 +331,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="_-* #,##0.00\ &quot;₫&quot;_-;\-* #,##0.00\ &quot;₫&quot;_-;_-* &quot;-&quot;??\ &quot;₫&quot;_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="_-* #,##0.00\ &quot;₫&quot;_-;\-* #,##0.00\ &quot;₫&quot;_-;_-* &quot;-&quot;??\ &quot;₫&quot;_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -351,13 +357,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
@@ -366,6 +365,14 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -385,6 +392,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="13"/>
       <color theme="3"/>
@@ -401,9 +415,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -417,19 +439,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -441,16 +462,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -464,6 +477,22 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
@@ -472,30 +501,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -522,187 +528,187 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -713,69 +719,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -797,8 +740,56 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -813,151 +804,166 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1275,7 +1281,7 @@
         <v>9</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G3" s="2">
         <v>1</v>
@@ -1286,10 +1292,10 @@
         <v>1003</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D4" s="4">
         <v>279000</v>
@@ -1309,19 +1315,19 @@
         <v>1004</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="4">
         <v>349000</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G5" s="2">
         <v>1</v>
@@ -1332,10 +1338,10 @@
         <v>1005</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="4">
         <v>244300</v>
@@ -1355,10 +1361,10 @@
         <v>1006</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" s="4">
         <v>399000</v>
@@ -1378,10 +1384,10 @@
         <v>1007</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D8" s="4">
         <v>399000</v>
@@ -1390,7 +1396,7 @@
         <v>9</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G8" s="2">
         <v>1</v>
@@ -1401,19 +1407,19 @@
         <v>1008</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D9" s="4">
         <v>499000</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="G9" s="2">
         <v>1</v>
@@ -1424,16 +1430,16 @@
         <v>1009</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D10" s="4">
         <v>499000</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>10</v>
@@ -1447,16 +1453,16 @@
         <v>1010</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D11" s="4">
         <v>599000</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>10</v>
@@ -1470,19 +1476,19 @@
         <v>1011</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D12" s="4">
         <v>599000</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="G12" s="2">
         <v>1</v>
@@ -1493,16 +1499,16 @@
         <v>1012</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D13" s="4">
         <v>419300</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>10</v>
@@ -1516,16 +1522,16 @@
         <v>1013</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D14" s="4">
         <v>549000</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>10</v>
@@ -1539,19 +1545,19 @@
         <v>1014</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D15" s="4">
         <v>419000</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G15" s="2">
         <v>1</v>
@@ -1562,16 +1568,16 @@
         <v>1015</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D16" s="4">
         <v>419300</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>10</v>
@@ -1585,16 +1591,16 @@
         <v>1016</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D17" s="4">
         <v>419300</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>10</v>
@@ -1608,16 +1614,16 @@
         <v>1017</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D18" s="4">
         <v>384000</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>10</v>
@@ -1631,19 +1637,19 @@
         <v>1018</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D19" s="4">
         <v>394000</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G19" s="2">
         <v>1</v>
@@ -1654,16 +1660,16 @@
         <v>1019</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D20" s="4">
         <v>499000</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>10</v>
@@ -1677,16 +1683,16 @@
         <v>1020</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D21" s="4">
         <v>599000</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>10</v>
@@ -1700,16 +1706,16 @@
         <v>1021</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D22" s="4">
         <v>419300</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>10</v>
@@ -1723,19 +1729,19 @@
         <v>1022</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D23" s="4">
         <v>599000</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G23" s="2">
         <v>1</v>
@@ -1746,16 +1752,16 @@
         <v>1023</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D24" s="4">
         <v>419300</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>10</v>
@@ -1769,16 +1775,16 @@
         <v>1024</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D25" s="4">
         <v>419300</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>10</v>
@@ -1792,16 +1798,16 @@
         <v>1025</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D26" s="4">
         <v>549000</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>10</v>
@@ -1815,19 +1821,19 @@
         <v>1026</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D27" s="4">
         <v>279000</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G27" s="2">
         <v>1</v>
@@ -1838,16 +1844,16 @@
         <v>1027</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D28" s="4">
         <v>419300</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>10</v>
@@ -1861,16 +1867,16 @@
         <v>1028</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D29" s="4">
         <v>179000</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>10</v>
@@ -1884,19 +1890,19 @@
         <v>1029</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D30" s="4">
         <v>419300</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G30" s="2">
         <v>1</v>
@@ -1907,16 +1913,16 @@
         <v>1030</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D31" s="4">
         <v>799000</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>10</v>
@@ -1930,19 +1936,19 @@
         <v>1031</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D32" s="4">
         <v>499000</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="G32" s="2">
         <v>1</v>
@@ -1953,19 +1959,19 @@
         <v>1032</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D33" s="4">
         <v>419300</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="G33" s="2">
         <v>1</v>
@@ -1976,16 +1982,16 @@
         <v>1033</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D34" s="4">
         <v>599000</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>10</v>
@@ -1999,16 +2005,16 @@
         <v>1034</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D35" s="4">
         <v>699000</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>10</v>
@@ -2022,19 +2028,19 @@
         <v>1035</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D36" s="4">
         <v>419300</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G36" s="2">
         <v>1</v>
@@ -2045,16 +2051,16 @@
         <v>1036</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D37" s="4">
         <v>699000</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>10</v>
@@ -2068,16 +2074,16 @@
         <v>1037</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D38" s="4">
         <v>524000</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>10</v>
@@ -2091,19 +2097,19 @@
         <v>1038</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D39" s="4">
         <v>2999000</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="G39" s="2">
         <v>1</v>
@@ -2114,19 +2120,19 @@
         <v>1039</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D40" s="4">
         <v>1199200</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G40" s="2">
         <v>1</v>
@@ -2137,19 +2143,19 @@
         <v>1040</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D41" s="4">
         <v>899000</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="G41" s="2">
         <v>1</v>
@@ -2176,10 +2182,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -2187,7 +2193,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -2195,7 +2201,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -2203,7 +2209,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -2211,7 +2217,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -2219,7 +2225,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>